<commit_message>
[Mutasi] - update multibin template
</commit_message>
<xml_diff>
--- a/public/upload/template/mutation_multi_bin_template.xlsx
+++ b/public/upload/template/mutation_multi_bin_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\test\Multibin Mutasi\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEF950ED-32B3-41EC-8D29-571A1E95D9BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FE5424B-ACAF-4153-B6F8-BC79DC179914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4225B295-9A20-4B2F-A3BB-F1C43B77D00E}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
   <si>
     <t>SKU</t>
   </si>
@@ -70,6 +70,15 @@
   </si>
   <si>
     <t>GL3-KAV9-A4-2</t>
+  </si>
+  <si>
+    <t>NOTES</t>
+  </si>
+  <si>
+    <t>DEFECT</t>
+  </si>
+  <si>
+    <t>REJECT</t>
   </si>
 </sst>
 </file>
@@ -422,7 +431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E6C4101-2C1D-4D07-8644-E2D15AC45FD2}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
@@ -431,7 +440,7 @@
     <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -444,8 +453,11 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -458,8 +470,11 @@
       <c r="D2">
         <v>2</v>
       </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -472,8 +487,11 @@
       <c r="D3">
         <v>3</v>
       </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -487,7 +505,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>

</xml_diff>